<commit_message>
auto update fantasy data
</commit_message>
<xml_diff>
--- a/IPL_Fantasy_Points.xlsx
+++ b/IPL_Fantasy_Points.xlsx
@@ -1335,19 +1335,19 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>357</v>
+        <v>400</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>357</v>
+        <v>400</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>357</v>
+        <v>400</v>
       </c>
     </row>
     <row r="22">
@@ -2367,19 +2367,19 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>48</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46">
@@ -2441,15 +2441,15 @@
           <t>BOWL</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>lokesh rahul</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>lockie ferguson</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>no_stats_yet</t>
+          <t>exact/alias</t>
         </is>
       </c>
       <c r="G47" t="n">
@@ -2883,19 +2883,19 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>232</v>
+        <v>248</v>
       </c>
     </row>
     <row r="58">
@@ -3614,19 +3614,19 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>287</v>
+        <v>346</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>287</v>
+        <v>346</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
       </c>
       <c r="K74" t="n">
-        <v>287</v>
+        <v>346</v>
       </c>
     </row>
     <row r="75">
@@ -3657,19 +3657,19 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>254</v>
+        <v>283</v>
       </c>
     </row>
     <row r="76">
@@ -4001,19 +4001,19 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="J83" t="n">
         <v>0</v>
       </c>
       <c r="K83" t="n">
-        <v>240</v>
+        <v>270</v>
       </c>
     </row>
     <row r="84">
@@ -4047,16 +4047,16 @@
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I84" t="n">
         <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="K84" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
     </row>
     <row r="85">
@@ -4302,19 +4302,19 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>255</v>
+        <v>306</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>255</v>
+        <v>306</v>
       </c>
       <c r="J90" t="n">
         <v>0</v>
       </c>
       <c r="K90" t="n">
-        <v>255</v>
+        <v>306</v>
       </c>
     </row>
     <row r="91">
@@ -4388,19 +4388,19 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>279</v>
+        <v>309</v>
       </c>
       <c r="H92" t="n">
         <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>279</v>
+        <v>309</v>
       </c>
       <c r="J92" t="n">
         <v>0</v>
       </c>
       <c r="K92" t="n">
-        <v>279</v>
+        <v>309</v>
       </c>
     </row>
     <row r="93">
@@ -4732,19 +4732,19 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="H100" t="n">
         <v>2</v>
       </c>
       <c r="I100" t="n">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="J100" t="n">
         <v>40</v>
       </c>
       <c r="K100" t="n">
-        <v>128</v>
+        <v>157</v>
       </c>
     </row>
     <row r="101">
@@ -5036,16 +5036,16 @@
         <v>3</v>
       </c>
       <c r="H107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I107" t="n">
         <v>0</v>
       </c>
       <c r="J107" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="K107" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
     </row>
     <row r="108">
@@ -5420,19 +5420,19 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="H116" t="n">
         <v>1</v>
       </c>
       <c r="I116" t="n">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="J116" t="n">
         <v>20</v>
       </c>
       <c r="K116" t="n">
-        <v>150</v>
+        <v>202</v>
       </c>
     </row>
     <row r="117">
@@ -6916,7 +6916,7 @@
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>suyash sharma</t>
+          <t>suryansh shedge</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -7057,16 +7057,16 @@
         <v>13</v>
       </c>
       <c r="H154" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I154" t="n">
         <v>13</v>
       </c>
       <c r="J154" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="K154" t="n">
-        <v>273</v>
+        <v>293</v>
       </c>
     </row>
     <row r="155">
@@ -7143,16 +7143,16 @@
         <v>0</v>
       </c>
       <c r="H156" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I156" t="n">
         <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="K156" t="n">
-        <v>80</v>
+        <v>140</v>
       </c>
     </row>
     <row r="157">
@@ -7902,15 +7902,15 @@
           <t>BOWL</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>jasprit bumrah</t>
-        </is>
-      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>harpreet brar</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>no_stats_yet</t>
+          <t>exact/alias</t>
         </is>
       </c>
       <c r="G174" t="n">
@@ -8185,7 +8185,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2664</v>
+        <v>2802</v>
       </c>
     </row>
     <row r="3">
@@ -8198,7 +8198,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2312</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="4">
@@ -8207,11 +8207,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AMEY11</t>
+          <t>NAKUL11</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2017</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="5">
@@ -8220,11 +8220,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BABA11</t>
+          <t>AMEY11</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1985</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="6">
@@ -8233,11 +8233,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NAKUL11</t>
+          <t>SKY11</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1974</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="7">
@@ -8246,11 +8246,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SKY11</t>
+          <t>BABA11</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1953</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="8">
@@ -8272,11 +8272,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HARSH11</t>
+          <t>VATSAL11</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1748</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="10">
@@ -8285,11 +8285,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>VATSAL11</t>
+          <t>HARSH11</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1693</v>
+        <v>1748</v>
       </c>
     </row>
     <row r="11">
@@ -8316,7 +8316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C170"/>
+  <dimension ref="A1:C174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8528,7 +8528,7 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -8707,7 +8707,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -8742,11 +8742,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>david miller</t>
+          <t>dasun shanaka</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
@@ -8755,50 +8755,50 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>david payne</t>
+          <t>david miller</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6</v>
+        <v>123</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>deepak chahar</t>
+          <t>david payne</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>6</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>devdutt padikkal</t>
+          <t>deepak chahar</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>242</v>
+        <v>6</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>dewald brevis</t>
+          <t>devdutt padikkal</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>64</v>
+        <v>242</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
@@ -8807,11 +8807,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>dhruv chand jurel</t>
+          <t>dewald brevis</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>232</v>
+        <v>64</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -8820,37 +8820,37 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>digvesh rathi</t>
+          <t>dhruv chand jurel</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>248</v>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>dilshan madushanka</t>
+          <t>digvesh rathi</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>donavon ferreira</t>
+          <t>dilshan madushanka</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="C41" t="n">
         <v>1</v>
@@ -8859,89 +8859,89 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>dushmantha chameera</t>
+          <t>donavon ferreira</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>eshan malinga</t>
+          <t>dushmantha chameera</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>finn allen</t>
+          <t>eshan malinga</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>george linde</t>
+          <t>finn allen</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>glenn phillips</t>
+          <t>george linde</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>gurjapneet singh</t>
+          <t>glenn phillips</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>hardik pandya</t>
+          <t>gurjapneet singh</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
         <v>3</v>
@@ -8950,24 +8950,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>harsh dubey</t>
+          <t>hardik pandya</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="C49" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>harshal patel</t>
+          <t>harpreet brar</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
         <v>0</v>
@@ -8976,24 +8976,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>heinrich klaasen</t>
+          <t>harsh dubey</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>349</v>
+        <v>13</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>himmat singh</t>
+          <t>harshal patel</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="C52" t="n">
         <v>0</v>
@@ -9002,11 +9002,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ishan kishan</t>
+          <t>heinrich klaasen</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>312</v>
+        <v>349</v>
       </c>
       <c r="C53" t="n">
         <v>0</v>
@@ -9015,11 +9015,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>jacob bethell</t>
+          <t>himmat singh</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C54" t="n">
         <v>0</v>
@@ -9028,102 +9028,102 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>jacob duffy</t>
+          <t>ishan kishan</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="C55" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>jamie overton</t>
+          <t>jacob bethell</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>136</v>
+        <v>34</v>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>jason holder</t>
+          <t>jacob duffy</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>jasprit bumrah</t>
+          <t>jamie overton</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>7</v>
+        <v>136</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>jaydev unadkat</t>
+          <t>jason holder</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>jitesh sharma</t>
+          <t>jasprit bumrah</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>jofra archer</t>
+          <t>jaydev unadkat</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C61" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>jos buttler</t>
+          <t>jitesh sharma</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>270</v>
+        <v>62</v>
       </c>
       <c r="C62" t="n">
         <v>0</v>
@@ -9132,63 +9132,63 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>josh hazlewood</t>
+          <t>jofra archer</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>kagiso rabada</t>
+          <t>jos buttler</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>35</v>
+        <v>270</v>
       </c>
       <c r="C64" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>kartik sharma</t>
+          <t>josh hazlewood</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>kartik tyagi</t>
+          <t>kagiso rabada</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>karun nair</t>
+          <t>kartik sharma</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
@@ -9197,24 +9197,24 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>khaleel ahmed</t>
+          <t>kartik tyagi</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>krish bhagat</t>
+          <t>karun nair</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
@@ -9223,63 +9223,63 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>krunal pandya</t>
+          <t>khaleel ahmed</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>kuldeep yadav</t>
+          <t>krish bhagat</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C71" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>kumar kushagra</t>
+          <t>krunal pandya</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>kyle jamieson</t>
+          <t>kuldeep yadav</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>lhuan dre pretorius</t>
+          <t>kumar kushagra</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
@@ -9288,24 +9288,24 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>liam livingstone</t>
+          <t>kyle jamieson</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>lokesh rahul</t>
+          <t>lhuan dre pretorius</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>358</v>
+        <v>0</v>
       </c>
       <c r="C76" t="n">
         <v>0</v>
@@ -9314,102 +9314,102 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>lungi ngidi</t>
+          <t>liam livingstone</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C77" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>manav suthar</t>
+          <t>lockie ferguson</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>manimaran siddharth</t>
+          <t>lokesh rahul</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0</v>
+        <v>358</v>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>marco jansen</t>
+          <t>lungi ngidi</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C80" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>marcus stoinis</t>
+          <t>manav suthar</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>matt henry</t>
+          <t>manimaran siddharth</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>matt short</t>
+          <t>marco jansen</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>mayank markande</t>
+          <t>marcus stoinis</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
@@ -9418,24 +9418,24 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>mayank rawat</t>
+          <t>matt henry</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C85" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>mayank yadav</t>
+          <t>matt short</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
@@ -9444,11 +9444,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>mitchell marsh</t>
+          <t>mayank markande</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>212</v>
+        <v>0</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -9457,128 +9457,128 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>mitchell santner</t>
+          <t>mayank rawat</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>mohammed shami</t>
+          <t>mayank yadav</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C89" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>mohammed siraj</t>
+          <t>mitchell marsh</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0</v>
+        <v>212</v>
       </c>
       <c r="C90" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>mohsin khan</t>
+          <t>mitchell santner</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="C91" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>mukesh choudhary</t>
+          <t>mohammed shami</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C92" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>mukesh kumar</t>
+          <t>mohammed siraj</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>0</v>
       </c>
       <c r="C93" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>mukul choudhary</t>
+          <t>mohsin khan</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="C94" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>naman dhir</t>
+          <t>mukesh choudhary</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>nandre burger</t>
+          <t>mukesh kumar</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C96" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>navdeep saini</t>
+          <t>mukul choudhary</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="C97" t="n">
         <v>0</v>
@@ -9587,11 +9587,11 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>nehal wadhera</t>
+          <t>naman dhir</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>65</v>
+        <v>154</v>
       </c>
       <c r="C98" t="n">
         <v>0</v>
@@ -9600,37 +9600,37 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>nicholas pooran</t>
+          <t>nandre burger</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="C99" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>nitish kumar reddy</t>
+          <t>navdeep saini</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>nitish rana</t>
+          <t>nehal wadhera</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>169</v>
+        <v>65</v>
       </c>
       <c r="C101" t="n">
         <v>0</v>
@@ -9639,37 +9639,37 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>noor ahmad</t>
+          <t>nicholas pooran</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="C102" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>pat cummins</t>
+          <t>nitish kumar reddy</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>pathum nissanka</t>
+          <t>nitish rana</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="C104" t="n">
         <v>0</v>
@@ -9678,50 +9678,50 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>philip salt</t>
+          <t>noor ahmad</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>202</v>
+        <v>10</v>
       </c>
       <c r="C105" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>prabhsimran singh</t>
+          <t>pat cummins</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>287</v>
+        <v>0</v>
       </c>
       <c r="C106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>praful hinge</t>
+          <t>pathum nissanka</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="C107" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>prashant veer</t>
+          <t>philip salt</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>49</v>
+        <v>202</v>
       </c>
       <c r="C108" t="n">
         <v>0</v>
@@ -9730,37 +9730,37 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>prasidh krishna</t>
+          <t>prabhsimran singh</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0</v>
+        <v>346</v>
       </c>
       <c r="C109" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>prince yadav</t>
+          <t>praful hinge</t>
         </is>
       </c>
       <c r="B110" t="n">
         <v>0</v>
       </c>
       <c r="C110" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>priyansh arya</t>
+          <t>prashant veer</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>254</v>
+        <v>49</v>
       </c>
       <c r="C111" t="n">
         <v>0</v>
@@ -9769,37 +9769,37 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>quinton de kock</t>
+          <t>prasidh krishna</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>rahul chahar</t>
+          <t>prince yadav</t>
         </is>
       </c>
       <c r="B113" t="n">
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>rahul tewatia</t>
+          <t>priyansh arya</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>49</v>
+        <v>283</v>
       </c>
       <c r="C114" t="n">
         <v>0</v>
@@ -9808,11 +9808,11 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>rajat patidar</t>
+          <t>quinton de kock</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>238</v>
+        <v>132</v>
       </c>
       <c r="C115" t="n">
         <v>0</v>
@@ -9821,115 +9821,115 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ramandeep singh</t>
+          <t>rahul chahar</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>rashid khan</t>
+          <t>rahul tewatia</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C117" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>rasikh salam</t>
+          <t>rajat patidar</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="C118" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ravi bishnoi</t>
+          <t>ramandeep singh</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="C119" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ravindra jadeja</t>
+          <t>rashid khan</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>132</v>
+        <v>28</v>
       </c>
       <c r="C120" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>rinku singh</t>
+          <t>rasikh salam</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="C121" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>rishabh pant</t>
+          <t>ravi bishnoi</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="C122" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>riyan parag</t>
+          <t>ravindra jadeja</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>88</v>
+        <v>132</v>
       </c>
       <c r="C123" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>rohit sharma</t>
+          <t>rinku singh</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>137</v>
+        <v>215</v>
       </c>
       <c r="C124" t="n">
         <v>0</v>
@@ -9938,37 +9938,37 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>romario shepherd</t>
+          <t>rishabh pant</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>39</v>
+        <v>189</v>
       </c>
       <c r="C125" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>rovman powell</t>
+          <t>riyan parag</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ruturaj gaikwad</t>
+          <t>rohit sharma</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>178</v>
+        <v>137</v>
       </c>
       <c r="C127" t="n">
         <v>0</v>
@@ -9977,24 +9977,24 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ryan rickelton</t>
+          <t>romario shepherd</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>137</v>
+        <v>39</v>
       </c>
       <c r="C128" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>sahil parakh</t>
+          <t>rovman powell</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="C129" t="n">
         <v>0</v>
@@ -10003,24 +10003,24 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>sakib hussain</t>
+          <t>ruturaj gaikwad</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="C130" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>salil arora</t>
+          <t>ryan rickelton</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>63</v>
+        <v>137</v>
       </c>
       <c r="C131" t="n">
         <v>0</v>
@@ -10029,11 +10029,11 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>sameer rizvi</t>
+          <t>sahil parakh</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>209</v>
+        <v>0</v>
       </c>
       <c r="C132" t="n">
         <v>0</v>
@@ -10042,24 +10042,24 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>sandeep sharma</t>
+          <t>sakib hussain</t>
         </is>
       </c>
       <c r="B133" t="n">
         <v>0</v>
       </c>
       <c r="C133" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>sanju samson</t>
+          <t>salil arora</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>304</v>
+        <v>63</v>
       </c>
       <c r="C134" t="n">
         <v>0</v>
@@ -10068,11 +10068,11 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>sarfaraz khan</t>
+          <t>sameer rizvi</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>161</v>
+        <v>209</v>
       </c>
       <c r="C135" t="n">
         <v>0</v>
@@ -10081,24 +10081,24 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>shahbaz ahmed</t>
+          <t>sandeep sharma</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C136" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>shahrukh khan</t>
+          <t>sanju samson</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>35</v>
+        <v>304</v>
       </c>
       <c r="C137" t="n">
         <v>0</v>
@@ -10107,37 +10107,37 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>shardul thakur</t>
+          <t>sarfaraz khan</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="C138" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>shashank singh</t>
+          <t>shahbaz ahmed</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>sherfane rutherford</t>
+          <t>shahrukh khan</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="C140" t="n">
         <v>0</v>
@@ -10146,50 +10146,50 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>shimron hetmyer</t>
+          <t>shardul thakur</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="C141" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>shivam dube</t>
+          <t>shashank singh</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="C142" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>shivang kumar</t>
+          <t>sherfane rutherford</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>21</v>
+        <v>103</v>
       </c>
       <c r="C143" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>shreyas iyer</t>
+          <t>shimron hetmyer</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>279</v>
+        <v>72</v>
       </c>
       <c r="C144" t="n">
         <v>0</v>
@@ -10198,50 +10198,50 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>shubham badriprasad dubey</t>
+          <t>shivam dube</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>19</v>
+        <v>150</v>
       </c>
       <c r="C145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>shubman gill</t>
+          <t>shivang kumar</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>330</v>
+        <v>21</v>
       </c>
       <c r="C146" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>sunil narine</t>
+          <t>shreyas iyer</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>40</v>
+        <v>309</v>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>suryakumar yadav</t>
+          <t>shubham badriprasad dubey</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>157</v>
+        <v>50</v>
       </c>
       <c r="C148" t="n">
         <v>0</v>
@@ -10250,37 +10250,37 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>suyash sharma</t>
+          <t>shubman gill</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0</v>
+        <v>330</v>
       </c>
       <c r="C149" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>t natarajan</t>
+          <t>sunil narine</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>tilak varma</t>
+          <t>suryakumar yadav</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="C151" t="n">
         <v>0</v>
@@ -10289,11 +10289,11 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>tim david</t>
+          <t>suryansh shedge</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>183</v>
+        <v>3</v>
       </c>
       <c r="C152" t="n">
         <v>0</v>
@@ -10302,50 +10302,50 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>tim seifert</t>
+          <t>suyash sharma</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C153" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>travis head</t>
+          <t>t natarajan</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>186</v>
+        <v>1</v>
       </c>
       <c r="C154" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>trent boult</t>
+          <t>tilak varma</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>1</v>
+        <v>181</v>
       </c>
       <c r="C155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>tristan stubbs</t>
+          <t>tim david</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="C156" t="n">
         <v>0</v>
@@ -10354,24 +10354,24 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>tushar deshpande</t>
+          <t>tim seifert</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C157" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>urvil patel</t>
+          <t>travis head</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>4</v>
+        <v>186</v>
       </c>
       <c r="C158" t="n">
         <v>0</v>
@@ -10380,24 +10380,24 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>vaibhav arora</t>
+          <t>trent boult</t>
         </is>
       </c>
       <c r="B159" t="n">
         <v>1</v>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>vaibhav suryavanshi</t>
+          <t>tristan stubbs</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>357</v>
+        <v>201</v>
       </c>
       <c r="C160" t="n">
         <v>0</v>
@@ -10406,24 +10406,24 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>varun chakravarthy</t>
+          <t>tushar deshpande</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C161" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>venkatesh iyer</t>
+          <t>urvil patel</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C162" t="n">
         <v>0</v>
@@ -10432,89 +10432,89 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>vijaykumar vyshak</t>
+          <t>vaibhav arora</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C163" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>vipraj nigam</t>
+          <t>vaibhav suryavanshi</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>12</v>
+        <v>400</v>
       </c>
       <c r="C164" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>virat kohli</t>
+          <t>varun chakravarthy</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>351</v>
+        <v>0</v>
       </c>
       <c r="C165" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>washington sundar</t>
+          <t>venkatesh iyer</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>157</v>
+        <v>29</v>
       </c>
       <c r="C166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>xavier bartlett</t>
+          <t>vijaykumar vyshak</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>yash raj punja</t>
+          <t>vipraj nigam</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>yashasvi jaiswal</t>
+          <t>virat kohli</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>255</v>
+        <v>351</v>
       </c>
       <c r="C169" t="n">
         <v>0</v>
@@ -10523,14 +10523,66 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
+          <t>washington sundar</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>157</v>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>xavier bartlett</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>11</v>
+      </c>
+      <c r="C171" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>yash raj punja</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>0</v>
+      </c>
+      <c r="C172" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>yashasvi jaiswal</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>306</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
           <t>yuzvendra chahal</t>
         </is>
       </c>
-      <c r="B170" t="n">
-        <v>0</v>
-      </c>
-      <c r="C170" t="n">
-        <v>4</v>
+      <c r="B174" t="n">
+        <v>0</v>
+      </c>
+      <c r="C174" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -10544,7 +10596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10951,7 +11003,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lockie Ferguson</t>
+          <t>Adam Milne</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -10967,7 +11019,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>lokesh rahul</t>
+          <t>david miller</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -10994,23 +11046,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Adam Milne</t>
+          <t>Jos Inglis</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>VATSAL11</t>
+          <t>BABA11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>david miller</t>
+          <t>marcus stoinis</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -11037,7 +11089,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jos Inglis</t>
+          <t>Prithvi Shaw</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -11053,7 +11105,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>marcus stoinis</t>
+          <t>prasidh krishna</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -11080,7 +11132,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Prithvi Shaw</t>
+          <t>liam livingston</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -11090,13 +11142,13 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>prasidh krishna</t>
+          <t>liam livingstone</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -11123,7 +11175,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>liam livingston</t>
+          <t>rachin ravindra</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -11139,7 +11191,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>liam livingstone</t>
+          <t>rashid khan</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -11166,7 +11218,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rachin ravindra</t>
+          <t>Zeeshan Ansari</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -11176,13 +11228,13 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>rashid khan</t>
+          <t>eshan malinga</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -11209,7 +11261,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Zeeshan Ansari</t>
+          <t>Mitchell Starc</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -11225,7 +11277,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>eshan malinga</t>
+          <t>mitchell santner</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -11252,17 +11304,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mitchell Starc</t>
+          <t>Mitchel Owen</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BABA11</t>
+          <t>DIPESH11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -11295,7 +11347,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mitchel Owen</t>
+          <t>Auqib Dar</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -11305,13 +11357,13 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>mitchell santner</t>
+          <t>auqib nabi</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -11338,23 +11390,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Auqib Dar</t>
+          <t>Arshin Kulkarni</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DIPESH11</t>
+          <t>NAKUL11</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>auqib nabi</t>
+          <t>ashwani kumar</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -11381,7 +11433,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Arshin Kulkarni</t>
+          <t>Nishant Sindhu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -11391,13 +11443,13 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ashwani kumar</t>
+          <t>shashank singh</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -11424,7 +11476,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nishant Sindhu</t>
+          <t>Jayant Yadav</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -11440,7 +11492,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>shashank singh</t>
+          <t>mayank yadav</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -11467,7 +11519,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jayant Yadav</t>
+          <t>Ajay Mandal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -11483,7 +11535,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mayank yadav</t>
+          <t>rajat patidar</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -11510,7 +11562,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ajay Mandal</t>
+          <t>Will Jacks</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -11526,7 +11578,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>rajat patidar</t>
+          <t>mitchell marsh</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -11553,7 +11605,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Will Jacks</t>
+          <t>Matheesha Pathirana</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -11563,13 +11615,13 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mitchell marsh</t>
+          <t>eshan malinga</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -11596,7 +11648,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Matheesha Pathirana</t>
+          <t>Ben Dwarshuis</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -11612,7 +11664,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>eshan malinga</t>
+          <t>b sai sudharshan</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -11639,23 +11691,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ben Dwarshuis</t>
+          <t>Manish Pandey</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NAKUL11</t>
+          <t>SKY11</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>b sai sudharshan</t>
+          <t>hardik pandya</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -11682,7 +11734,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Manish Pandey</t>
+          <t>Arjun Tendulkar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -11692,13 +11744,13 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>hardik pandya</t>
+          <t>karun nair</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -11725,7 +11777,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Arjun Tendulkar</t>
+          <t>Kwena Maphaka</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -11741,7 +11793,7 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>karun nair</t>
+          <t>aiden markram</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -11768,23 +11820,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kwena Maphaka</t>
+          <t>Ramkrishna Ghosh</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SKY11</t>
+          <t>HARSH11</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>aiden markram</t>
+          <t>angkrish raghuvanshi</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -11811,7 +11863,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ramkrishna Ghosh</t>
+          <t>Azmatullah Omarzai</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -11821,13 +11873,13 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>angkrish raghuvanshi</t>
+          <t>mitchell marsh</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -11854,23 +11906,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Azmatullah Omarzai</t>
+          <t>akshat raghuwanshi</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HARSH11</t>
+          <t>AMEY11</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mitchell marsh</t>
+          <t>angkrish raghuvanshi</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -11897,7 +11949,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>akshat raghuwanshi</t>
+          <t>Suryansh Shegde</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -11913,7 +11965,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>angkrish raghuvanshi</t>
+          <t>suryansh shedge</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -11940,7 +11992,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Suryansh Shegde</t>
+          <t>Tejasvi Singh</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -11956,7 +12008,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>suyash sharma</t>
+          <t>prabhsimran singh</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -11983,7 +12035,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tejasvi Singh</t>
+          <t>Sai Kishor</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -11993,13 +12045,13 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>BOWL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>prabhsimran singh</t>
+          <t>ishan kishan</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -12026,7 +12078,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sai Kishor</t>
+          <t>Akash Deep</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -12042,7 +12094,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ishan kishan</t>
+          <t>arshdeep singh</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -12069,23 +12121,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Akash Deep</t>
+          <t>Ben Duckett</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AMEY11</t>
+          <t>PRATIK11</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BOWL</t>
+          <t>BAT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>arshdeep singh</t>
+          <t>ryan rickelton</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -12112,7 +12164,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ben Duckett</t>
+          <t>Rahul Tripathi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -12128,7 +12180,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ryan rickelton</t>
+          <t>rahul tewatia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -12155,7 +12207,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rahul Tripathi</t>
+          <t>Dre Pretorius</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -12171,7 +12223,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>rahul tewatia</t>
+          <t>lhuan dre pretorius</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -12198,7 +12250,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Dre Pretorius</t>
+          <t>Matthew Breetzke</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -12214,7 +12266,7 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>lhuan dre pretorius</t>
+          <t>matt henry</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -12241,7 +12293,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Matthew Breetzke</t>
+          <t>Anuj Rawat</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -12257,7 +12309,7 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>matt henry</t>
+          <t>mayank rawat</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -12284,7 +12336,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Anuj Rawat</t>
+          <t>Wanindu Hasaranga</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -12294,13 +12346,13 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BAT</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>mayank rawat</t>
+          <t>sandeep sharma</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -12321,92 +12373,6 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Wanindu Hasaranga</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>PRATIK11</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>sandeep sharma</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>no_stats_yet</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Harpreet Brar</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>PRATIK11</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>BOWL</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>jasprit bumrah</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>no_stats_yet</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12580,19 +12546,19 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="J2" t="n">
         <v>20</v>
       </c>
       <c r="K2" t="n">
-        <v>150</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">

</xml_diff>